<commit_message>
Fix: orden consecutivo natural por número de categoría en egresos y reportes
</commit_message>
<xml_diff>
--- a/data/adonai_data_completo.xlsx
+++ b/data/adonai_data_completo.xlsx
@@ -2648,7 +2648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -2680,195 +2680,6 @@
       <c r="E1" s="6" t="inlineStr">
         <is>
           <t>responsable</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2505165</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>juliet</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>15152123</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2025-09-05</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>202020</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>juliet dayana</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>20202010</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2025-09-09</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>505050</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>maria jose</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>12135351</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>5050505</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>dasdas</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>20202010</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2025-09-15</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2323</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>maria jose</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>20202010</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2025-12-15</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>576345634</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>juliet dayana</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>57554</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>0045-05-04</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>45546546</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>dasdas</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>20202020</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>admin</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.77734375" customWidth="1" min="3" max="3"/>
@@ -3031,256 +2842,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-09-14</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>banco</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ingresos</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Administrativo</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Intereses bancarios</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>20202040</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>fdsfsd</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>200000</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-09-17</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>caja</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>ingresos</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Misión Institucional</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Donaciones USA</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>505050</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>fdsfsd</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09-14</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>caja</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ingresos</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Otros ingresos</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Otros ingresos</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>base</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>200000</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>banco</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ingresos</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Administrativo</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Donaciones SRL</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>ughghjgkjgkj</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>caja</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ingresos</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Misión Institucional</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Donaciones específicas locales</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Cita m</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>600000</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>caja</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ingresos</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Misión Institucional</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Donaciones USA</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>base</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360"/>
@@ -3293,7 +2854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="18.33203125" customWidth="1" min="3" max="3"/>
@@ -3347,171 +2908,6 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Responsable</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-12-14</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>banco</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>egresos</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>10. Misional Madres</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Transporte</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>505050</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>base</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>caja</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>egresos</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>5. Redes Sociales</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>ughghjgkjgkj</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>banco</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>egresos</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1. Nómina</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Dirección General</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>otro</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>4999999.95</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>banco</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>egresos</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1. Nómina</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Prestamos</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>fdsfsd</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>admin</t>
         </is>
       </c>
     </row>
@@ -3570,7 +2966,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -3580,7 +2976,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10519999.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -3590,7 +2986,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-6519999.949999999</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3604,7 +3000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.5546875" customWidth="1" min="1" max="1"/>
@@ -3684,102 +3080,6 @@
         <is>
           <t>Balance</t>
         </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2400000</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2400000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D4" t="n">
-        <v>-20000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-5000000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C6" t="n">
-        <v>5499999.95</v>
-      </c>
-      <c r="D6" t="n">
-        <v>-4999999.95</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>600000</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>600000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>500000</v>
       </c>
     </row>
   </sheetData>
@@ -3851,7 +3151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3906,16 +3206,6 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-12</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>4500</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>